<commit_message>
phase3A: complete dataset diagnostics before training
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R120e57e6097d4046"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R4469b8965d7a48c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="3" r:id="R7fbe3cdfb0a1499f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rdb7d966a131341ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9c82191b3e544d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R67b807ea945b4115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="3" r:id="Rb7ece5b5954e4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rbab37de7860c4251"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2265,7 +2265,7 @@
       </x:c>
       <x:c r="B4" s="2" t="n">
         <x:f>COUNTIF(Checklist!$F:$F,"Chưa làm")</x:f>
-        <x:v>300</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
         <x:v>4</x:v>
@@ -2301,7 +2301,7 @@
       </x:c>
       <x:c r="B6" s="2" t="n">
         <x:f>COUNTIF(Checklist!$F:$F,"Hoàn thành")</x:f>
-        <x:v>231</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
         <x:v>10</x:v>
@@ -2337,7 +2337,7 @@
       </x:c>
       <x:c r="B8" s="5" t="n">
         <x:f>IFERROR(B6/B3,0)</x:f>
-        <x:v>0.4333958724202627</x:v>
+        <x:v>0.4652908067542214</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
         <x:v>16</x:v>
@@ -2539,7 +2539,7 @@
       </x:c>
       <x:c r="C16" t="n">
         <x:f>'Phase Summary'!C6</x:f>
-        <x:v>17</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D16" t="n">
         <x:f>'Phase Summary'!D6</x:f>
@@ -2547,7 +2547,7 @@
       </x:c>
       <x:c r="E16" t="n">
         <x:f>'Phase Summary'!E6</x:f>
-        <x:v>0</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F16" t="n">
         <x:f>'Phase Summary'!F6</x:f>
@@ -2559,7 +2559,7 @@
       </x:c>
       <x:c r="H16" s="6" t="n">
         <x:f>'Phase Summary'!H6</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -11403,8 +11403,8 @@
       <x:c r="E237" s="10" t="s">
         <x:v>301</x:v>
       </x:c>
-      <x:c r="F237" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F237" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G237" s="10" t="s">
         <x:v>60</x:v>
@@ -11414,11 +11414,15 @@
       </x:c>
       <x:c r="I237" s="10"/>
       <x:c r="J237" s="10"/>
-      <x:c r="K237" s="10"/>
-      <x:c r="L237" s="10"/>
-      <x:c r="M237" s="10">
+      <x:c r="K237" s="10" t="str">
+        <x:v>PASS: fixed-train class distribution đã hoàn tất; 14 detection classes; image-level support là primary rarity measure.</x:v>
+      </x:c>
+      <x:c r="L237" s="10" t="str">
+        <x:v>plots/dataset/class_distribution.png; reports/03A_class_distribution.csv; reports/03A_class_imbalance.csv</x:v>
+      </x:c>
+      <x:c r="M237" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="238" ht="27.600000381469727">
@@ -11437,8 +11441,8 @@
       <x:c r="E238" s="10" t="s">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="F238" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F238" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G238" s="10" t="s">
         <x:v>60</x:v>
@@ -11448,11 +11452,15 @@
       </x:c>
       <x:c r="I238" s="10"/>
       <x:c r="J238" s="10"/>
-      <x:c r="K238" s="10"/>
-      <x:c r="L238" s="10"/>
-      <x:c r="M238" s="10">
+      <x:c r="K238" s="10" t="str">
+        <x:v>PASS: bbox annotation count theo class đã thống kê; giữ tách biệt với image-level support và không diễn giải là unique clinical lesions.</x:v>
+      </x:c>
+      <x:c r="L238" s="10" t="str">
+        <x:v>reports/03A_class_distribution.csv; plots/dataset/class_distribution.png</x:v>
+      </x:c>
+      <x:c r="M238" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="27.600000381469727">
@@ -11471,8 +11479,8 @@
       <x:c r="E239" s="10" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="F239" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F239" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G239" s="10" t="s">
         <x:v>60</x:v>
@@ -11482,11 +11490,15 @@
       </x:c>
       <x:c r="I239" s="10"/>
       <x:c r="J239" s="10"/>
-      <x:c r="K239" s="10"/>
-      <x:c r="L239" s="10"/>
-      <x:c r="M239" s="10">
+      <x:c r="K239" s="10" t="str">
+        <x:v>PASS: normalized-area bbox distribution đã hoàn tất; Small/Medium/Large = 37.10% / 57.85% / 5.05%; primary thresholds 0.01/0.10 giữ nguyên.</x:v>
+      </x:c>
+      <x:c r="L239" s="10" t="str">
+        <x:v>plots/dataset/bbox_distribution.png; reports/03A_bbox_distribution.csv; reports/03A_bbox_summary.csv; reports/03A_threshold_sensitivity.csv</x:v>
+      </x:c>
+      <x:c r="M239" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="27.600000381469727">
@@ -11505,8 +11517,8 @@
       <x:c r="E240" s="10" t="s">
         <x:v>304</x:v>
       </x:c>
-      <x:c r="F240" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F240" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G240" s="10" t="s">
         <x:v>60</x:v>
@@ -11516,11 +11528,15 @@
       </x:c>
       <x:c r="I240" s="10"/>
       <x:c r="J240" s="10"/>
-      <x:c r="K240" s="10"/>
-      <x:c r="L240" s="10"/>
-      <x:c r="M240" s="10">
+      <x:c r="K240" s="10" t="str">
+        <x:v>PASS: bbox-centre heatmap 50×50, annotation-weighted, fixed train; chỉ mô tả spatial annotation distribution.</x:v>
+      </x:c>
+      <x:c r="L240" s="10" t="str">
+        <x:v>plots/dataset/bbox_location_heatmap.png; reports/dataset_analysis_report.md</x:v>
+      </x:c>
+      <x:c r="M240" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="241" ht="27.600000381469727">
@@ -11539,8 +11555,8 @@
       <x:c r="E241" s="10" t="s">
         <x:v>305</x:v>
       </x:c>
-      <x:c r="F241" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F241" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G241" s="10" t="s">
         <x:v>60</x:v>
@@ -11550,11 +11566,15 @@
       </x:c>
       <x:c r="I241" s="10"/>
       <x:c r="J241" s="10"/>
-      <x:c r="K241" s="10"/>
-      <x:c r="L241" s="10"/>
-      <x:c r="M241" s="10">
+      <x:c r="K241" s="10" t="str">
+        <x:v>PASS: rare operational definition khóa trước diagnostics: image prevalence &lt;5%; rare classes = Atelectasis (130; 3.79%) và Pneumothorax (66; 1.93%).</x:v>
+      </x:c>
+      <x:c r="L241" s="10" t="str">
+        <x:v>configs/protocol/phase3A_dataset_diagnostics.yaml; reports/03A_class_distribution.csv; reports/03A_threshold_sensitivity.csv; reports/dataset_analysis_report.md</x:v>
+      </x:c>
+      <x:c r="M241" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="27.600000381469727">
@@ -11573,8 +11593,8 @@
       <x:c r="E242" s="10" t="s">
         <x:v>306</x:v>
       </x:c>
-      <x:c r="F242" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F242" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G242" s="10" t="s">
         <x:v>60</x:v>
@@ -11584,11 +11604,15 @@
       </x:c>
       <x:c r="I242" s="10"/>
       <x:c r="J242" s="10"/>
-      <x:c r="K242" s="10"/>
-      <x:c r="L242" s="10"/>
-      <x:c r="M242" s="10">
+      <x:c r="K242" s="10" t="str">
+        <x:v>PASS: fixed train có 350/3426 No Finding = 10.216%; No Finding là zero-GT negative image, không phải detection class.</x:v>
+      </x:c>
+      <x:c r="L242" s="10" t="str">
+        <x:v>plots/dataset/negative_image_distribution.png; reports/03A_negative_distribution.csv</x:v>
+      </x:c>
+      <x:c r="M242" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="243" ht="27.600000381469727">
@@ -11607,8 +11631,8 @@
       <x:c r="E243" s="10" t="s">
         <x:v>307</x:v>
       </x:c>
-      <x:c r="F243" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F243" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G243" s="10" t="s">
         <x:v>60</x:v>
@@ -11618,11 +11642,15 @@
       </x:c>
       <x:c r="I243" s="10"/>
       <x:c r="J243" s="10"/>
-      <x:c r="K243" s="10"/>
-      <x:c r="L243" s="10"/>
-      <x:c r="M243" s="10">
+      <x:c r="K243" s="10" t="str">
+        <x:v>PASS: train/val/test structural distribution đã đối chiếu; detailed diagnostics không mở trên val/test.</x:v>
+      </x:c>
+      <x:c r="L243" s="10" t="str">
+        <x:v>reports/03A_split_distribution.csv; reports/03A_dataset_diagnostics_validation.json</x:v>
+      </x:c>
+      <x:c r="M243" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="244" ht="27.600000381469727">
@@ -11641,8 +11669,8 @@
       <x:c r="E244" s="10" t="s">
         <x:v>308</x:v>
       </x:c>
-      <x:c r="F244" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F244" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G244" s="10" t="s">
         <x:v>60</x:v>
@@ -11652,11 +11680,15 @@
       </x:c>
       <x:c r="I244" s="10"/>
       <x:c r="J244" s="10"/>
-      <x:c r="K244" s="10"/>
-      <x:c r="L244" s="10"/>
-      <x:c r="M244" s="10">
+      <x:c r="K244" s="10" t="str">
+        <x:v>PASS: detailed scopes chỉ gồm train + labeled 1/5/10/20%; val/test structural-only; hidden unlabeled GT không được dùng; sensitivity không dùng để retune threshold.</x:v>
+      </x:c>
+      <x:c r="L244" s="10" t="str">
+        <x:v>reports/03A_dataset_diagnostics_validation.json; configs/protocol/phase3A_dataset_diagnostics.yaml</x:v>
+      </x:c>
+      <x:c r="M244" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="245" ht="27.600000381469727">
@@ -11675,8 +11707,8 @@
       <x:c r="E245" s="10" t="s">
         <x:v>309</x:v>
       </x:c>
-      <x:c r="F245" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F245" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G245" s="10" t="s">
         <x:v>60</x:v>
@@ -11686,11 +11718,15 @@
       </x:c>
       <x:c r="I245" s="10"/>
       <x:c r="J245" s="10"/>
-      <x:c r="K245" s="10"/>
-      <x:c r="L245" s="10"/>
-      <x:c r="M245" s="10">
+      <x:c r="K245" s="10" t="str">
+        <x:v>OUTPUT VERIFIED: final pre-training report đã review claim discipline và regenerate sau wording fix; Phase 3A researcher/GPT closure = CLOSED/PASS.</x:v>
+      </x:c>
+      <x:c r="L245" s="10" t="str">
+        <x:v>reports/dataset_analysis_report.md; reports/03A_dataset_diagnostics_validation.json; reports/03A_artifact_manifest.json; reports/03A_guardrails_junit.xml</x:v>
+      </x:c>
+      <x:c r="M245" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="246" ht="27.600000381469727">
@@ -11709,8 +11745,8 @@
       <x:c r="E246" s="10" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="F246" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F246" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G246" s="10" t="s">
         <x:v>60</x:v>
@@ -11720,11 +11756,15 @@
       </x:c>
       <x:c r="I246" s="10"/>
       <x:c r="J246" s="10"/>
-      <x:c r="K246" s="10"/>
-      <x:c r="L246" s="10"/>
-      <x:c r="M246" s="10">
+      <x:c r="K246" s="10" t="str">
+        <x:v>OUTPUT VERIFIED: class distribution figure sinh từ fixed train; đi kèm machine-readable class distribution/imbalance CSV.</x:v>
+      </x:c>
+      <x:c r="L246" s="10" t="str">
+        <x:v>plots/dataset/class_distribution.png; reports/03A_class_distribution.csv</x:v>
+      </x:c>
+      <x:c r="M246" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="247" ht="27.600000381469727">
@@ -11743,8 +11783,8 @@
       <x:c r="E247" s="10" t="s">
         <x:v>311</x:v>
       </x:c>
-      <x:c r="F247" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F247" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G247" s="10" t="s">
         <x:v>60</x:v>
@@ -11754,11 +11794,15 @@
       </x:c>
       <x:c r="I247" s="10"/>
       <x:c r="J247" s="10"/>
-      <x:c r="K247" s="10"/>
-      <x:c r="L247" s="10"/>
-      <x:c r="M247" s="10">
+      <x:c r="K247" s="10" t="str">
+        <x:v>OUTPUT VERIFIED: bbox distribution figure gồm continuous normalized-area distribution và locked Small/Medium/Large categories.</x:v>
+      </x:c>
+      <x:c r="L247" s="10" t="str">
+        <x:v>plots/dataset/bbox_distribution.png; reports/03A_bbox_distribution.csv; reports/03A_bbox_summary.csv</x:v>
+      </x:c>
+      <x:c r="M247" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="248" ht="27.600000381469727">
@@ -11777,8 +11821,8 @@
       <x:c r="E248" s="10" t="s">
         <x:v>312</x:v>
       </x:c>
-      <x:c r="F248" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F248" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G248" s="10" t="s">
         <x:v>60</x:v>
@@ -11788,11 +11832,15 @@
       </x:c>
       <x:c r="I248" s="10"/>
       <x:c r="J248" s="10"/>
-      <x:c r="K248" s="10"/>
-      <x:c r="L248" s="10"/>
-      <x:c r="M248" s="10">
+      <x:c r="K248" s="10" t="str">
+        <x:v>OUTPUT VERIFIED: 50×50 annotation-weighted bbox-centre heatmap; không claim unique clinical lesion density.</x:v>
+      </x:c>
+      <x:c r="L248" s="10" t="str">
+        <x:v>plots/dataset/bbox_location_heatmap.png; reports/dataset_analysis_report.md</x:v>
+      </x:c>
+      <x:c r="M248" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="27.600000381469727">
@@ -11811,8 +11859,8 @@
       <x:c r="E249" s="10" t="s">
         <x:v>313</x:v>
       </x:c>
-      <x:c r="F249" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F249" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G249" s="10" t="s">
         <x:v>60</x:v>
@@ -11822,11 +11870,15 @@
       </x:c>
       <x:c r="I249" s="10"/>
       <x:c r="J249" s="10"/>
-      <x:c r="K249" s="10"/>
-      <x:c r="L249" s="10"/>
-      <x:c r="M249" s="10">
+      <x:c r="K249" s="10" t="str">
+        <x:v>OUTPUT VERIFIED: positive vs No Finding/zero-GT fixed-train distribution; 3076 positive và 350 negative.</x:v>
+      </x:c>
+      <x:c r="L249" s="10" t="str">
+        <x:v>plots/dataset/negative_image_distribution.png; reports/03A_negative_distribution.csv</x:v>
+      </x:c>
+      <x:c r="M249" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="250" ht="27.600000381469727">
@@ -11845,8 +11897,8 @@
       <x:c r="E250" s="10" t="s">
         <x:v>314</x:v>
       </x:c>
-      <x:c r="F250" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F250" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G250" s="10" t="s">
         <x:v>60</x:v>
@@ -11856,11 +11908,15 @@
       </x:c>
       <x:c r="I250" s="10"/>
       <x:c r="J250" s="10"/>
-      <x:c r="K250" s="10"/>
-      <x:c r="L250" s="10"/>
-      <x:c r="M250" s="10">
+      <x:c r="K250" s="10" t="str">
+        <x:v>PASS: báo cáo pre-training hoàn tất trước bất kỳ model training nào; guardrails cuối 53/53 PASS; full run hard_error_count=0, warning_count=0.</x:v>
+      </x:c>
+      <x:c r="L250" s="10" t="str">
+        <x:v>reports/dataset_analysis_report.md; reports/03A_guardrails_junit.xml; reports/03A_dataset_diagnostics_validation.json</x:v>
+      </x:c>
+      <x:c r="M250" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="251" ht="27.600000381469727">
@@ -11879,8 +11935,8 @@
       <x:c r="E251" s="10" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="F251" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F251" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G251" s="10" t="s">
         <x:v>60</x:v>
@@ -11890,11 +11946,15 @@
       </x:c>
       <x:c r="I251" s="10"/>
       <x:c r="J251" s="10"/>
-      <x:c r="K251" s="10"/>
-      <x:c r="L251" s="10"/>
-      <x:c r="M251" s="10">
+      <x:c r="K251" s="10" t="str">
+        <x:v>PASS: rare classes theo locked &lt;5% rule = Atelectasis và Pneumothorax; rare status là dataset-level low support, không phải clinical rarity.</x:v>
+      </x:c>
+      <x:c r="L251" s="10" t="str">
+        <x:v>reports/03A_class_distribution.csv; reports/03A_threshold_sensitivity.csv; reports/dataset_analysis_report.md</x:v>
+      </x:c>
+      <x:c r="M251" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="252" ht="27.600000381469727">
@@ -11913,8 +11973,8 @@
       <x:c r="E252" s="10" t="s">
         <x:v>316</x:v>
       </x:c>
-      <x:c r="F252" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F252" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G252" s="10" t="s">
         <x:v>60</x:v>
@@ -11924,11 +11984,15 @@
       </x:c>
       <x:c r="I252" s="10"/>
       <x:c r="J252" s="10"/>
-      <x:c r="K252" s="10"/>
-      <x:c r="L252" s="10"/>
-      <x:c r="M252" s="10">
+      <x:c r="K252" s="10" t="str">
+        <x:v>PASS: image-support imbalance ratio max/min = 32.48; CV = 0.8025. Labeled budgets giữ 14/14 class coverage nhưng 1% chỉ có 1 image cho mỗi rare class.</x:v>
+      </x:c>
+      <x:c r="L252" s="10" t="str">
+        <x:v>reports/03A_class_imbalance.csv; reports/03A_labeled_budget_coverage.csv; reports/03A_label_cardinality.csv; reports/03A_class_cooccurrence.csv</x:v>
+      </x:c>
+      <x:c r="M252" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="253" ht="27.600000381469727">
@@ -11947,8 +12011,8 @@
       <x:c r="E253" s="10" t="s">
         <x:v>317</x:v>
       </x:c>
-      <x:c r="F253" s="10" t="s">
-        <x:v>3</x:v>
+      <x:c r="F253" s="10" t="str">
+        <x:v>Hoàn thành</x:v>
       </x:c>
       <x:c r="G253" s="10" t="s">
         <x:v>60</x:v>
@@ -11958,11 +12022,15 @@
       </x:c>
       <x:c r="I253" s="10"/>
       <x:c r="J253" s="10"/>
-      <x:c r="K253" s="10"/>
-      <x:c r="L253" s="10"/>
-      <x:c r="M253" s="10">
+      <x:c r="K253" s="10" t="str">
+        <x:v>PASS: bbox normalized-area categories = Small 37.10%, Medium 57.85%, Large 5.05%; sensitivity là SECONDARY/NON-GATING và không đổi primary thresholds.</x:v>
+      </x:c>
+      <x:c r="L253" s="10" t="str">
+        <x:v>reports/03A_bbox_distribution.csv; reports/03A_bbox_summary.csv; reports/03A_threshold_sensitivity.csv; plots/dataset/bbox_distribution.png</x:v>
+      </x:c>
+      <x:c r="M253" s="10" t="n">
         <x:f t="shared" si="3"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="254" ht="27.600000381469727">
@@ -26838,7 +26906,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc0a0192908049bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5fe4a224d54516"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27019,7 +27087,7 @@
       </x:c>
       <x:c r="C6" t="n">
         <x:f>COUNTIFS(Checklist!$B:$B,A6,Checklist!$F:$F,"Chưa làm")</x:f>
-        <x:v>17</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" t="n">
         <x:f>COUNTIFS(Checklist!$B:$B,A6,Checklist!$F:$F,"Đang làm")</x:f>
@@ -27027,7 +27095,7 @@
       </x:c>
       <x:c r="E6" t="n">
         <x:f>COUNTIFS(Checklist!$B:$B,A6,Checklist!$F:$F,"Hoàn thành")</x:f>
-        <x:v>0</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F6" t="n">
         <x:f>COUNTIFS(Checklist!$B:$B,A6,Checklist!$F:$F,"Bị chặn")</x:f>
@@ -27039,7 +27107,7 @@
       </x:c>
       <x:c r="H6" s="6" t="n">
         <x:f t="shared" si="0">IFERROR(E6/B6,0)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -27311,7 +27379,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3081555325344bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b10ca77510e41ef"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>

<commit_message>
close Gate I and freeze implementation inputs
</commit_message>
<xml_diff>
--- a/CHECKLIST_TRIEN_KHAI_FULL.xlsx
+++ b/CHECKLIST_TRIEN_KHAI_FULL.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R9c82191b3e544d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R67b807ea945b4115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="3" r:id="Rb7ece5b5954e4b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="Rbab37de7860c4251"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R107eb9f1edec435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R6545d842859d4684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="3" r:id="Ra6c351618219438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" r:id="R3954e60eb295491e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -976,9 +976,6 @@
     <x:t xml:space="preserve">4A.0 Full-label supervised upper bound</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Chọn detector chính.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Train trên 100% labeled train.</x:t>
   </x:si>
   <x:si>
@@ -992,9 +989,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Không thay đổi tiêu chí chọn checkpoint giữa các experiment.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Evaluate trên fixed test set.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Lưu config, seed, RNG state, checkpoint, log.</x:t>
@@ -12046,8 +12040,8 @@
       <x:c r="D254" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E254" s="10" t="s">
-        <x:v>319</x:v>
+      <x:c r="E254" s="10" t="str">
+        <x:v>Triển khai cả hai official architectures: Faster R-CNN ResNet-50/FPN và Faster R-CNN Swin-T/FPN; không model-shopping.</x:v>
       </x:c>
       <x:c r="F254" s="10" t="s">
         <x:v>3</x:v>
@@ -12060,8 +12054,13 @@
       </x:c>
       <x:c r="I254" s="10"/>
       <x:c r="J254" s="10"/>
-      <x:c r="K254" s="10"/>
-      <x:c r="L254" s="10"/>
+      <x:c r="K254" s="10" t="str">
+        <x:v>DOCUMENTATION DRIFT CORRECTED AT GATE I: MASTER D4-A khóa cả R50 và Swin-T là official architectures.</x:v>
+      </x:c>
+      <x:c r="L254" s="10" t="str">
+        <x:v>MASTER_D1_D7_FINAL_IMPLEMENTATION_CONTRACT_VI.md::D4-A
+vietluanvan.md::D4-A</x:v>
+      </x:c>
       <x:c r="M254" s="10">
         <x:f t="shared" si="3"/>
         <x:v>0</x:v>
@@ -12081,7 +12080,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E255" s="10" t="s">
-        <x:v>320</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="F255" s="10" t="s">
         <x:v>3</x:v>
@@ -12115,7 +12114,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E256" s="10" t="s">
-        <x:v>321</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="F256" s="10" t="s">
         <x:v>3</x:v>
@@ -12149,7 +12148,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E257" s="10" t="s">
-        <x:v>322</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="F257" s="10" t="s">
         <x:v>3</x:v>
@@ -12183,7 +12182,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E258" s="10" t="s">
-        <x:v>323</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="F258" s="10" t="s">
         <x:v>3</x:v>
@@ -12217,7 +12216,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E259" s="10" t="s">
-        <x:v>324</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F259" s="10" t="s">
         <x:v>3</x:v>
@@ -12250,8 +12249,8 @@
       <x:c r="D260" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E260" s="10" t="s">
-        <x:v>325</x:v>
+      <x:c r="E260" s="10" t="str">
+        <x:v>Không evaluate fixed test trong Phase 4; chỉ final-test campaign sau khi toàn bộ authorization gates được khóa và PASS.</x:v>
       </x:c>
       <x:c r="F260" s="10" t="s">
         <x:v>3</x:v>
@@ -12264,8 +12263,12 @@
       </x:c>
       <x:c r="I260" s="10"/>
       <x:c r="J260" s="10"/>
-      <x:c r="K260" s="10"/>
-      <x:c r="L260" s="10"/>
+      <x:c r="K260" s="10" t="str">
+        <x:v>DOCUMENTATION DRIFT CORRECTED AT GATE I: Phase 4 dùng validation-only checkpoint selection; test vẫn đóng đến frozen final-test campaign.</x:v>
+      </x:c>
+      <x:c r="L260" s="10" t="str">
+        <x:v>MASTER_D1_D7_FINAL_IMPLEMENTATION_CONTRACT_VI.md::Test firewall/Gate sequence</x:v>
+      </x:c>
       <x:c r="M260" s="10">
         <x:f t="shared" si="4"/>
         <x:v>0</x:v>
@@ -12285,7 +12288,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="E261" s="10" t="s">
-        <x:v>326</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="F261" s="10" t="s">
         <x:v>3</x:v>
@@ -12316,10 +12319,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D262" s="10" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="E262" s="10" t="s">
-        <x:v>328</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="F262" s="10" t="s">
         <x:v>3</x:v>
@@ -12350,10 +12353,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D263" s="10" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="E263" s="10" t="s">
         <x:v>327</x:v>
-      </x:c>
-      <x:c r="E263" s="10" t="s">
-        <x:v>329</x:v>
       </x:c>
       <x:c r="F263" s="10" t="s">
         <x:v>3</x:v>
@@ -12384,10 +12387,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D264" s="10" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="E264" s="10" t="s">
-        <x:v>330</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="F264" s="10" t="s">
         <x:v>3</x:v>
@@ -12418,10 +12421,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D265" s="10" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="E265" s="10" t="s">
-        <x:v>331</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="F265" s="10" t="s">
         <x:v>3</x:v>
@@ -12452,10 +12455,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D266" s="10" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="E266" s="10" t="s">
-        <x:v>332</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="F266" s="10" t="s">
         <x:v>3</x:v>
@@ -12486,10 +12489,10 @@
         <x:v>318</x:v>
       </x:c>
       <x:c r="D267" s="10" t="s">
-        <x:v>327</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="E267" s="10" t="s">
-        <x:v>333</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="F267" s="10" t="s">
         <x:v>3</x:v>
@@ -12523,7 +12526,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="E268" s="10" t="s">
-        <x:v>334</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="F268" s="10" t="s">
         <x:v>3</x:v>
@@ -12557,7 +12560,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="E269" s="10" t="s">
-        <x:v>335</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="F269" s="10" t="s">
         <x:v>3</x:v>
@@ -12591,7 +12594,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="E270" s="10" t="s">
-        <x:v>336</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="F270" s="10" t="s">
         <x:v>3</x:v>
@@ -12625,7 +12628,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E271" s="10" t="s">
-        <x:v>337</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="F271" s="10" t="s">
         <x:v>3</x:v>
@@ -12659,7 +12662,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E272" s="10" t="s">
-        <x:v>338</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="F272" s="10" t="s">
         <x:v>3</x:v>
@@ -12693,7 +12696,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E273" s="10" t="s">
-        <x:v>339</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="F273" s="10" t="s">
         <x:v>3</x:v>
@@ -12727,7 +12730,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E274" s="10" t="s">
-        <x:v>340</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="F274" s="10" t="s">
         <x:v>3</x:v>
@@ -12761,7 +12764,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="E275" s="10" t="s">
-        <x:v>341</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="F275" s="10" t="s">
         <x:v>3</x:v>
@@ -12789,13 +12792,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C276" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D276" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E276" s="10" t="s">
-        <x:v>343</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="F276" s="10" t="s">
         <x:v>3</x:v>
@@ -12823,13 +12826,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C277" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D277" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E277" s="10" t="s">
-        <x:v>344</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="F277" s="10" t="s">
         <x:v>3</x:v>
@@ -12857,13 +12860,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C278" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D278" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E278" s="10" t="s">
-        <x:v>345</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="F278" s="10" t="s">
         <x:v>3</x:v>
@@ -12891,13 +12894,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C279" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D279" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E279" s="10" t="s">
-        <x:v>346</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="F279" s="10" t="s">
         <x:v>3</x:v>
@@ -12925,7 +12928,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C280" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D280" s="10" t="s">
         <x:v>58</x:v>
@@ -12959,7 +12962,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C281" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D281" s="10" t="s">
         <x:v>58</x:v>
@@ -12993,13 +12996,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C282" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D282" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E282" s="10" t="s">
-        <x:v>347</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="F282" s="10" t="s">
         <x:v>3</x:v>
@@ -13027,13 +13030,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C283" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D283" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E283" s="10" t="s">
-        <x:v>348</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="F283" s="10" t="s">
         <x:v>3</x:v>
@@ -13061,13 +13064,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C284" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D284" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E284" s="10" t="s">
-        <x:v>349</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="F284" s="10" t="s">
         <x:v>3</x:v>
@@ -13095,13 +13098,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C285" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D285" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E285" s="10" t="s">
-        <x:v>350</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="F285" s="10" t="s">
         <x:v>3</x:v>
@@ -13129,13 +13132,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C286" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D286" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E286" s="10" t="s">
-        <x:v>351</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="F286" s="10" t="s">
         <x:v>3</x:v>
@@ -13163,13 +13166,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C287" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D287" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E287" s="10" t="s">
-        <x:v>352</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="F287" s="10" t="s">
         <x:v>3</x:v>
@@ -13197,13 +13200,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C288" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D288" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E288" s="10" t="s">
-        <x:v>353</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="F288" s="10" t="s">
         <x:v>3</x:v>
@@ -13231,7 +13234,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C289" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D289" s="10" t="s">
         <x:v>80</x:v>
@@ -13265,7 +13268,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C290" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D290" s="10" t="s">
         <x:v>80</x:v>
@@ -13299,13 +13302,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C291" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D291" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E291" s="10" t="s">
-        <x:v>354</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="F291" s="10" t="s">
         <x:v>3</x:v>
@@ -13333,13 +13336,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C292" s="10" t="s">
-        <x:v>342</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="D292" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E292" s="10" t="s">
-        <x:v>355</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="F292" s="10" t="s">
         <x:v>3</x:v>
@@ -13367,13 +13370,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C293" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D293" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E293" s="10" t="s">
-        <x:v>357</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="F293" s="10" t="s">
         <x:v>3</x:v>
@@ -13401,13 +13404,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C294" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D294" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E294" s="10" t="s">
-        <x:v>358</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="F294" s="10" t="s">
         <x:v>3</x:v>
@@ -13435,13 +13438,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C295" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D295" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E295" s="10" t="s">
-        <x:v>359</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="F295" s="10" t="s">
         <x:v>3</x:v>
@@ -13469,13 +13472,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C296" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D296" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E296" s="10" t="s">
-        <x:v>360</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="F296" s="10" t="s">
         <x:v>3</x:v>
@@ -13503,13 +13506,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C297" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D297" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E297" s="10" t="s">
-        <x:v>361</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="F297" s="10" t="s">
         <x:v>3</x:v>
@@ -13537,13 +13540,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C298" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D298" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E298" s="10" t="s">
-        <x:v>362</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="F298" s="10" t="s">
         <x:v>3</x:v>
@@ -13571,13 +13574,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C299" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D299" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E299" s="10" t="s">
-        <x:v>363</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="F299" s="10" t="s">
         <x:v>3</x:v>
@@ -13605,13 +13608,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="C300" s="10" t="s">
-        <x:v>356</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="D300" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E300" s="10" t="s">
-        <x:v>364</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="F300" s="10" t="s">
         <x:v>3</x:v>
@@ -13639,13 +13642,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C301" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D301" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E301" s="10" t="s">
-        <x:v>366</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="F301" s="10" t="s">
         <x:v>3</x:v>
@@ -13673,13 +13676,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C302" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D302" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E302" s="10" t="s">
-        <x:v>367</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="F302" s="10" t="s">
         <x:v>3</x:v>
@@ -13707,13 +13710,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C303" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D303" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E303" s="10" t="s">
-        <x:v>368</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="F303" s="10" t="s">
         <x:v>3</x:v>
@@ -13741,13 +13744,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C304" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D304" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E304" s="10" t="s">
-        <x:v>369</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="F304" s="10" t="s">
         <x:v>3</x:v>
@@ -13775,13 +13778,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C305" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D305" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E305" s="10" t="s">
-        <x:v>370</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="F305" s="10" t="s">
         <x:v>3</x:v>
@@ -13809,13 +13812,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C306" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D306" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E306" s="10" t="s">
-        <x:v>371</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="F306" s="10" t="s">
         <x:v>3</x:v>
@@ -13843,13 +13846,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C307" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D307" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E307" s="10" t="s">
-        <x:v>372</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="F307" s="10" t="s">
         <x:v>3</x:v>
@@ -13877,13 +13880,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C308" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D308" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E308" s="10" t="s">
-        <x:v>373</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="F308" s="10" t="s">
         <x:v>3</x:v>
@@ -13911,13 +13914,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C309" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D309" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E309" s="10" t="s">
-        <x:v>350</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="F309" s="10" t="s">
         <x:v>3</x:v>
@@ -13945,13 +13948,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C310" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D310" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E310" s="10" t="s">
-        <x:v>374</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F310" s="10" t="s">
         <x:v>3</x:v>
@@ -13979,13 +13982,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C311" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D311" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E311" s="10" t="s">
-        <x:v>375</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="F311" s="10" t="s">
         <x:v>3</x:v>
@@ -14013,13 +14016,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C312" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D312" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E312" s="10" t="s">
-        <x:v>376</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="F312" s="10" t="s">
         <x:v>3</x:v>
@@ -14047,13 +14050,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C313" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D313" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E313" s="10" t="s">
-        <x:v>377</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="F313" s="10" t="s">
         <x:v>3</x:v>
@@ -14081,13 +14084,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C314" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D314" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E314" s="10" t="s">
-        <x:v>378</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="F314" s="10" t="s">
         <x:v>3</x:v>
@@ -14115,13 +14118,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C315" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D315" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E315" s="10" t="s">
-        <x:v>379</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="F315" s="10" t="s">
         <x:v>3</x:v>
@@ -14149,13 +14152,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C316" s="10" t="s">
-        <x:v>365</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D316" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E316" s="10" t="s">
-        <x:v>380</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="F316" s="10" t="s">
         <x:v>3</x:v>
@@ -14183,13 +14186,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C317" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D317" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E317" s="10" t="s">
-        <x:v>382</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="F317" s="10" t="s">
         <x:v>3</x:v>
@@ -14217,13 +14220,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C318" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D318" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E318" s="10" t="s">
-        <x:v>383</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="F318" s="10" t="s">
         <x:v>3</x:v>
@@ -14251,13 +14254,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C319" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D319" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E319" s="10" t="s">
-        <x:v>384</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="F319" s="10" t="s">
         <x:v>3</x:v>
@@ -14285,13 +14288,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C320" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D320" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E320" s="10" t="s">
-        <x:v>385</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="F320" s="10" t="s">
         <x:v>3</x:v>
@@ -14319,13 +14322,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C321" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D321" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E321" s="10" t="s">
-        <x:v>386</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="F321" s="10" t="s">
         <x:v>3</x:v>
@@ -14353,13 +14356,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C322" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D322" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E322" s="10" t="s">
-        <x:v>387</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="F322" s="10" t="s">
         <x:v>3</x:v>
@@ -14387,13 +14390,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C323" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D323" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E323" s="10" t="s">
-        <x:v>388</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="F323" s="10" t="s">
         <x:v>3</x:v>
@@ -14421,13 +14424,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C324" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D324" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E324" s="10" t="s">
-        <x:v>389</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="F324" s="10" t="s">
         <x:v>3</x:v>
@@ -14455,13 +14458,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C325" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D325" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E325" s="10" t="s">
-        <x:v>390</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="F325" s="10" t="s">
         <x:v>3</x:v>
@@ -14489,13 +14492,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C326" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D326" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E326" s="10" t="s">
-        <x:v>391</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="F326" s="10" t="s">
         <x:v>3</x:v>
@@ -14523,13 +14526,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C327" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D327" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E327" s="10" t="s">
-        <x:v>392</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="F327" s="10" t="s">
         <x:v>3</x:v>
@@ -14557,13 +14560,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C328" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D328" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E328" s="10" t="s">
-        <x:v>393</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="F328" s="10" t="s">
         <x:v>3</x:v>
@@ -14591,13 +14594,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C329" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D329" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E329" s="10" t="s">
-        <x:v>394</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="F329" s="10" t="s">
         <x:v>3</x:v>
@@ -14625,13 +14628,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C330" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D330" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E330" s="10" t="s">
-        <x:v>395</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="F330" s="10" t="s">
         <x:v>3</x:v>
@@ -14659,13 +14662,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C331" s="10" t="s">
-        <x:v>381</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="D331" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E331" s="10" t="s">
-        <x:v>396</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="F331" s="10" t="s">
         <x:v>3</x:v>
@@ -14693,13 +14696,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C332" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D332" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E332" s="10" t="s">
-        <x:v>398</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="F332" s="10" t="s">
         <x:v>3</x:v>
@@ -14727,13 +14730,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C333" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D333" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E333" s="10" t="s">
-        <x:v>399</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="F333" s="10" t="s">
         <x:v>3</x:v>
@@ -14761,13 +14764,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C334" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D334" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E334" s="10" t="s">
-        <x:v>400</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="F334" s="10" t="s">
         <x:v>3</x:v>
@@ -14795,13 +14798,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C335" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D335" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E335" s="10" t="s">
-        <x:v>401</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="F335" s="10" t="s">
         <x:v>3</x:v>
@@ -14829,13 +14832,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C336" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D336" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E336" s="10" t="s">
-        <x:v>402</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="F336" s="10" t="s">
         <x:v>3</x:v>
@@ -14863,13 +14866,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C337" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D337" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E337" s="10" t="s">
-        <x:v>403</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="F337" s="10" t="s">
         <x:v>3</x:v>
@@ -14897,13 +14900,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C338" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D338" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E338" s="10" t="s">
-        <x:v>404</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F338" s="10" t="s">
         <x:v>3</x:v>
@@ -14931,13 +14934,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C339" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D339" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E339" s="10" t="s">
-        <x:v>405</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="F339" s="10" t="s">
         <x:v>3</x:v>
@@ -14965,13 +14968,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C340" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D340" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E340" s="10" t="s">
-        <x:v>406</x:v>
+        <x:v>404</x:v>
       </x:c>
       <x:c r="F340" s="10" t="s">
         <x:v>3</x:v>
@@ -14999,13 +15002,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C341" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D341" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E341" s="10" t="s">
-        <x:v>407</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="F341" s="10" t="s">
         <x:v>3</x:v>
@@ -15033,13 +15036,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C342" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D342" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E342" s="10" t="s">
-        <x:v>408</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="F342" s="10" t="s">
         <x:v>3</x:v>
@@ -15067,13 +15070,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C343" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D343" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E343" s="10" t="s">
-        <x:v>409</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="F343" s="10" t="s">
         <x:v>3</x:v>
@@ -15101,13 +15104,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C344" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D344" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E344" s="10" t="s">
-        <x:v>410</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="F344" s="10" t="s">
         <x:v>3</x:v>
@@ -15135,13 +15138,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C345" s="10" t="s">
-        <x:v>397</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="D345" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E345" s="10" t="s">
-        <x:v>411</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="F345" s="10" t="s">
         <x:v>3</x:v>
@@ -15169,13 +15172,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C346" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D346" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E346" s="10" t="s">
-        <x:v>413</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="F346" s="10" t="s">
         <x:v>3</x:v>
@@ -15203,13 +15206,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C347" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D347" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E347" s="10" t="s">
-        <x:v>414</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="F347" s="10" t="s">
         <x:v>3</x:v>
@@ -15237,13 +15240,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C348" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D348" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E348" s="10" t="s">
-        <x:v>415</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="F348" s="10" t="s">
         <x:v>3</x:v>
@@ -15271,13 +15274,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C349" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D349" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E349" s="10" t="s">
-        <x:v>416</x:v>
+        <x:v>414</x:v>
       </x:c>
       <x:c r="F349" s="10" t="s">
         <x:v>3</x:v>
@@ -15305,13 +15308,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C350" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D350" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E350" s="10" t="s">
-        <x:v>417</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="F350" s="10" t="s">
         <x:v>3</x:v>
@@ -15339,13 +15342,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C351" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D351" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E351" s="10" t="s">
-        <x:v>418</x:v>
+        <x:v>416</x:v>
       </x:c>
       <x:c r="F351" s="10" t="s">
         <x:v>3</x:v>
@@ -15373,13 +15376,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C352" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D352" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E352" s="10" t="s">
-        <x:v>419</x:v>
+        <x:v>417</x:v>
       </x:c>
       <x:c r="F352" s="10" t="s">
         <x:v>3</x:v>
@@ -15407,13 +15410,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C353" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D353" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E353" s="10" t="s">
-        <x:v>420</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="F353" s="10" t="s">
         <x:v>3</x:v>
@@ -15441,13 +15444,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C354" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D354" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E354" s="10" t="s">
-        <x:v>421</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="F354" s="10" t="s">
         <x:v>3</x:v>
@@ -15475,13 +15478,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C355" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D355" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E355" s="10" t="s">
-        <x:v>422</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="F355" s="10" t="s">
         <x:v>3</x:v>
@@ -15509,13 +15512,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C356" s="10" t="s">
-        <x:v>412</x:v>
+        <x:v>410</x:v>
       </x:c>
       <x:c r="D356" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E356" s="10" t="s">
-        <x:v>423</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="F356" s="10" t="s">
         <x:v>3</x:v>
@@ -15543,13 +15546,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C357" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D357" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E357" s="10" t="s">
-        <x:v>425</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="F357" s="10" t="s">
         <x:v>3</x:v>
@@ -15577,13 +15580,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C358" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D358" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E358" s="10" t="s">
-        <x:v>426</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="F358" s="10" t="s">
         <x:v>3</x:v>
@@ -15611,13 +15614,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C359" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D359" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E359" s="10" t="s">
-        <x:v>427</x:v>
+        <x:v>425</x:v>
       </x:c>
       <x:c r="F359" s="10" t="s">
         <x:v>3</x:v>
@@ -15645,13 +15648,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C360" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D360" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E360" s="10" t="s">
-        <x:v>428</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="F360" s="10" t="s">
         <x:v>3</x:v>
@@ -15679,13 +15682,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C361" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D361" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E361" s="10" t="s">
-        <x:v>429</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="F361" s="10" t="s">
         <x:v>3</x:v>
@@ -15713,13 +15716,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C362" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D362" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E362" s="10" t="s">
-        <x:v>430</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="F362" s="10" t="s">
         <x:v>3</x:v>
@@ -15747,13 +15750,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C363" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D363" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E363" s="10" t="s">
-        <x:v>431</x:v>
+        <x:v>429</x:v>
       </x:c>
       <x:c r="F363" s="10" t="s">
         <x:v>3</x:v>
@@ -15781,13 +15784,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C364" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D364" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E364" s="10" t="s">
-        <x:v>432</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="F364" s="10" t="s">
         <x:v>3</x:v>
@@ -15815,13 +15818,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C365" s="10" t="s">
-        <x:v>424</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="D365" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E365" s="10" t="s">
-        <x:v>433</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="F365" s="10" t="s">
         <x:v>3</x:v>
@@ -15849,13 +15852,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C366" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D366" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E366" s="10" t="s">
-        <x:v>435</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="F366" s="10" t="s">
         <x:v>3</x:v>
@@ -15883,13 +15886,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C367" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D367" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E367" s="10" t="s">
-        <x:v>436</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="F367" s="10" t="s">
         <x:v>3</x:v>
@@ -15917,13 +15920,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C368" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D368" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E368" s="10" t="s">
-        <x:v>437</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="F368" s="10" t="s">
         <x:v>3</x:v>
@@ -15951,13 +15954,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C369" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D369" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E369" s="10" t="s">
-        <x:v>438</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="F369" s="10" t="s">
         <x:v>3</x:v>
@@ -15985,13 +15988,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C370" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D370" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E370" s="10" t="s">
-        <x:v>439</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="F370" s="10" t="s">
         <x:v>3</x:v>
@@ -16019,13 +16022,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C371" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D371" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E371" s="10" t="s">
-        <x:v>440</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="F371" s="10" t="s">
         <x:v>3</x:v>
@@ -16053,13 +16056,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C372" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D372" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E372" s="10" t="s">
-        <x:v>441</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="F372" s="10" t="s">
         <x:v>3</x:v>
@@ -16087,13 +16090,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C373" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D373" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E373" s="10" t="s">
-        <x:v>442</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="F373" s="10" t="s">
         <x:v>3</x:v>
@@ -16121,13 +16124,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C374" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D374" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E374" s="10" t="s">
-        <x:v>443</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F374" s="10" t="s">
         <x:v>3</x:v>
@@ -16155,13 +16158,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C375" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D375" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E375" s="10" t="s">
-        <x:v>444</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="F375" s="10" t="s">
         <x:v>3</x:v>
@@ -16189,13 +16192,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C376" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D376" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E376" s="10" t="s">
-        <x:v>445</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="F376" s="10" t="s">
         <x:v>3</x:v>
@@ -16223,13 +16226,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C377" s="10" t="s">
-        <x:v>434</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="D377" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E377" s="10" t="s">
-        <x:v>446</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="F377" s="10" t="s">
         <x:v>3</x:v>
@@ -16257,13 +16260,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C378" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D378" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E378" s="10" t="s">
-        <x:v>448</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F378" s="10" t="s">
         <x:v>3</x:v>
@@ -16291,13 +16294,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C379" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D379" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E379" s="10" t="s">
-        <x:v>449</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="F379" s="10" t="s">
         <x:v>3</x:v>
@@ -16325,13 +16328,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C380" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D380" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E380" s="10" t="s">
-        <x:v>450</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="F380" s="10" t="s">
         <x:v>3</x:v>
@@ -16359,13 +16362,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C381" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D381" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E381" s="10" t="s">
-        <x:v>451</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F381" s="10" t="s">
         <x:v>3</x:v>
@@ -16393,7 +16396,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C382" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D382" s="10" t="s">
         <x:v>58</x:v>
@@ -16427,7 +16430,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C383" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D383" s="10" t="s">
         <x:v>58</x:v>
@@ -16461,7 +16464,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C384" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D384" s="10" t="s">
         <x:v>58</x:v>
@@ -16495,13 +16498,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C385" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D385" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E385" s="10" t="s">
-        <x:v>452</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="F385" s="10" t="s">
         <x:v>3</x:v>
@@ -16529,13 +16532,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C386" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D386" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E386" s="10" t="s">
-        <x:v>453</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="F386" s="10" t="s">
         <x:v>3</x:v>
@@ -16563,13 +16566,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C387" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D387" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E387" s="10" t="s">
-        <x:v>374</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F387" s="10" t="s">
         <x:v>3</x:v>
@@ -16597,13 +16600,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C388" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D388" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E388" s="10" t="s">
-        <x:v>454</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F388" s="10" t="s">
         <x:v>3</x:v>
@@ -16631,13 +16634,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C389" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D389" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E389" s="10" t="s">
-        <x:v>455</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="F389" s="10" t="s">
         <x:v>3</x:v>
@@ -16665,13 +16668,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C390" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D390" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E390" s="10" t="s">
-        <x:v>456</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F390" s="10" t="s">
         <x:v>3</x:v>
@@ -16699,13 +16702,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C391" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D391" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E391" s="10" t="s">
-        <x:v>457</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="F391" s="10" t="s">
         <x:v>3</x:v>
@@ -16733,13 +16736,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C392" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D392" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E392" s="10" t="s">
-        <x:v>458</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="F392" s="10" t="s">
         <x:v>3</x:v>
@@ -16767,13 +16770,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C393" s="10" t="s">
-        <x:v>447</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="D393" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E393" s="10" t="s">
-        <x:v>459</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="F393" s="10" t="s">
         <x:v>3</x:v>
@@ -16801,13 +16804,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C394" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D394" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E394" s="10" t="s">
-        <x:v>461</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F394" s="10" t="s">
         <x:v>3</x:v>
@@ -16835,13 +16838,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C395" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D395" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E395" s="10" t="s">
-        <x:v>462</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="F395" s="10" t="s">
         <x:v>3</x:v>
@@ -16869,13 +16872,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C396" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D396" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E396" s="10" t="s">
-        <x:v>463</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="F396" s="10" t="s">
         <x:v>3</x:v>
@@ -16903,13 +16906,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C397" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D397" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E397" s="10" t="s">
-        <x:v>464</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="F397" s="10" t="s">
         <x:v>3</x:v>
@@ -16937,13 +16940,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C398" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D398" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E398" s="10" t="s">
-        <x:v>465</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="F398" s="10" t="s">
         <x:v>3</x:v>
@@ -16971,13 +16974,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C399" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D399" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E399" s="10" t="s">
-        <x:v>466</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="F399" s="10" t="s">
         <x:v>3</x:v>
@@ -17005,13 +17008,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C400" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D400" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E400" s="10" t="s">
-        <x:v>467</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="F400" s="10" t="s">
         <x:v>3</x:v>
@@ -17039,13 +17042,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C401" s="10" t="s">
-        <x:v>460</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="D401" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E401" s="10" t="s">
-        <x:v>468</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="F401" s="10" t="s">
         <x:v>3</x:v>
@@ -17073,13 +17076,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C402" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D402" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E402" s="10" t="s">
-        <x:v>470</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="F402" s="10" t="s">
         <x:v>3</x:v>
@@ -17107,13 +17110,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C403" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D403" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E403" s="10" t="s">
-        <x:v>471</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F403" s="10" t="s">
         <x:v>3</x:v>
@@ -17141,13 +17144,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C404" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D404" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E404" s="10" t="s">
-        <x:v>472</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="F404" s="10" t="s">
         <x:v>3</x:v>
@@ -17175,13 +17178,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C405" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D405" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E405" s="10" t="s">
-        <x:v>473</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="F405" s="10" t="s">
         <x:v>3</x:v>
@@ -17209,13 +17212,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C406" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D406" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E406" s="10" t="s">
-        <x:v>474</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="F406" s="10" t="s">
         <x:v>3</x:v>
@@ -17243,13 +17246,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C407" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D407" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E407" s="10" t="s">
-        <x:v>475</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="F407" s="10" t="s">
         <x:v>3</x:v>
@@ -17277,13 +17280,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C408" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D408" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E408" s="10" t="s">
-        <x:v>476</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="F408" s="10" t="s">
         <x:v>3</x:v>
@@ -17311,13 +17314,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C409" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D409" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E409" s="10" t="s">
-        <x:v>477</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="F409" s="10" t="s">
         <x:v>3</x:v>
@@ -17345,13 +17348,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C410" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D410" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E410" s="10" t="s">
-        <x:v>420</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="F410" s="10" t="s">
         <x:v>3</x:v>
@@ -17379,13 +17382,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C411" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D411" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E411" s="10" t="s">
-        <x:v>478</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="F411" s="10" t="s">
         <x:v>3</x:v>
@@ -17413,13 +17416,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C412" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D412" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E412" s="10" t="s">
-        <x:v>479</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="F412" s="10" t="s">
         <x:v>3</x:v>
@@ -17447,13 +17450,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C413" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D413" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E413" s="10" t="s">
-        <x:v>480</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="F413" s="10" t="s">
         <x:v>3</x:v>
@@ -17481,13 +17484,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C414" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D414" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E414" s="10" t="s">
-        <x:v>481</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="F414" s="10" t="s">
         <x:v>3</x:v>
@@ -17515,13 +17518,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C415" s="10" t="s">
-        <x:v>469</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D415" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E415" s="10" t="s">
-        <x:v>482</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F415" s="10" t="s">
         <x:v>3</x:v>
@@ -17549,13 +17552,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C416" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D416" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E416" s="10" t="s">
-        <x:v>484</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="F416" s="10" t="s">
         <x:v>3</x:v>
@@ -17583,13 +17586,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C417" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D417" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E417" s="10" t="s">
-        <x:v>485</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="F417" s="10" t="s">
         <x:v>3</x:v>
@@ -17617,13 +17620,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C418" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D418" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E418" s="10" t="s">
-        <x:v>486</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="F418" s="10" t="s">
         <x:v>3</x:v>
@@ -17651,13 +17654,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C419" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D419" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E419" s="10" t="s">
-        <x:v>487</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="F419" s="10" t="s">
         <x:v>3</x:v>
@@ -17685,13 +17688,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C420" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D420" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E420" s="10" t="s">
-        <x:v>488</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="F420" s="10" t="s">
         <x:v>3</x:v>
@@ -17719,13 +17722,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C421" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D421" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E421" s="10" t="s">
-        <x:v>489</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="F421" s="10" t="s">
         <x:v>3</x:v>
@@ -17753,13 +17756,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C422" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D422" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E422" s="10" t="s">
-        <x:v>490</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="F422" s="10" t="s">
         <x:v>3</x:v>
@@ -17787,13 +17790,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C423" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D423" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E423" s="10" t="s">
-        <x:v>491</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="F423" s="10" t="s">
         <x:v>3</x:v>
@@ -17821,13 +17824,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C424" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D424" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E424" s="10" t="s">
-        <x:v>492</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="F424" s="10" t="s">
         <x:v>3</x:v>
@@ -17855,13 +17858,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C425" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D425" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E425" s="10" t="s">
-        <x:v>493</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="F425" s="10" t="s">
         <x:v>3</x:v>
@@ -17889,13 +17892,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C426" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D426" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E426" s="10" t="s">
-        <x:v>494</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F426" s="10" t="s">
         <x:v>3</x:v>
@@ -17923,13 +17926,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C427" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D427" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E427" s="10" t="s">
-        <x:v>495</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F427" s="10" t="s">
         <x:v>3</x:v>
@@ -17957,13 +17960,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C428" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D428" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E428" s="10" t="s">
-        <x:v>496</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F428" s="10" t="s">
         <x:v>3</x:v>
@@ -17991,13 +17994,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C429" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D429" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E429" s="10" t="s">
-        <x:v>497</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="F429" s="10" t="s">
         <x:v>3</x:v>
@@ -18025,13 +18028,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C430" s="10" t="s">
-        <x:v>483</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D430" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E430" s="10" t="s">
-        <x:v>498</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="F430" s="10" t="s">
         <x:v>3</x:v>
@@ -18059,13 +18062,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C431" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D431" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E431" s="10" t="s">
-        <x:v>500</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="F431" s="10" t="s">
         <x:v>3</x:v>
@@ -18093,13 +18096,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C432" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D432" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E432" s="10" t="s">
-        <x:v>501</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="F432" s="10" t="s">
         <x:v>3</x:v>
@@ -18127,13 +18130,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C433" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D433" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E433" s="10" t="s">
-        <x:v>502</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="F433" s="10" t="s">
         <x:v>3</x:v>
@@ -18161,13 +18164,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C434" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D434" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E434" s="10" t="s">
-        <x:v>503</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="F434" s="10" t="s">
         <x:v>3</x:v>
@@ -18195,13 +18198,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C435" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D435" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E435" s="10" t="s">
-        <x:v>504</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="F435" s="10" t="s">
         <x:v>3</x:v>
@@ -18229,13 +18232,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C436" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D436" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E436" s="10" t="s">
-        <x:v>505</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="F436" s="10" t="s">
         <x:v>3</x:v>
@@ -18263,13 +18266,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C437" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D437" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E437" s="10" t="s">
-        <x:v>506</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F437" s="10" t="s">
         <x:v>3</x:v>
@@ -18297,13 +18300,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C438" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D438" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E438" s="10" t="s">
-        <x:v>507</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F438" s="10" t="s">
         <x:v>3</x:v>
@@ -18331,13 +18334,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C439" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D439" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E439" s="10" t="s">
-        <x:v>508</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="F439" s="10" t="s">
         <x:v>3</x:v>
@@ -18365,13 +18368,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C440" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D440" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E440" s="10" t="s">
-        <x:v>509</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="F440" s="10" t="s">
         <x:v>3</x:v>
@@ -18399,13 +18402,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C441" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D441" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E441" s="10" t="s">
-        <x:v>510</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="F441" s="10" t="s">
         <x:v>3</x:v>
@@ -18433,13 +18436,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C442" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D442" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E442" s="10" t="s">
-        <x:v>393</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="F442" s="10" t="s">
         <x:v>3</x:v>
@@ -18467,13 +18470,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C443" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D443" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E443" s="10" t="s">
-        <x:v>511</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="F443" s="10" t="s">
         <x:v>3</x:v>
@@ -18501,13 +18504,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C444" s="10" t="s">
-        <x:v>499</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="D444" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E444" s="10" t="s">
-        <x:v>512</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="F444" s="10" t="s">
         <x:v>3</x:v>
@@ -18535,13 +18538,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C445" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D445" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E445" s="10" t="s">
-        <x:v>514</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="F445" s="10" t="s">
         <x:v>3</x:v>
@@ -18569,7 +18572,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C446" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D446" s="10" t="s">
         <x:v>58</x:v>
@@ -18603,13 +18606,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C447" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D447" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E447" s="10" t="s">
-        <x:v>515</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="F447" s="10" t="s">
         <x:v>3</x:v>
@@ -18637,13 +18640,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C448" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D448" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E448" s="10" t="s">
-        <x:v>516</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="F448" s="10" t="s">
         <x:v>3</x:v>
@@ -18671,13 +18674,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C449" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D449" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E449" s="10" t="s">
-        <x:v>517</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="F449" s="10" t="s">
         <x:v>3</x:v>
@@ -18705,13 +18708,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C450" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D450" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E450" s="10" t="s">
-        <x:v>518</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="F450" s="10" t="s">
         <x:v>3</x:v>
@@ -18739,7 +18742,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C451" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D451" s="10" t="s">
         <x:v>58</x:v>
@@ -18773,13 +18776,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C452" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D452" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E452" s="10" t="s">
-        <x:v>519</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="F452" s="10" t="s">
         <x:v>3</x:v>
@@ -18807,13 +18810,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C453" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D453" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E453" s="10" t="s">
-        <x:v>520</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F453" s="10" t="s">
         <x:v>3</x:v>
@@ -18841,13 +18844,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C454" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D454" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E454" s="10" t="s">
-        <x:v>521</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="F454" s="10" t="s">
         <x:v>3</x:v>
@@ -18875,13 +18878,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C455" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D455" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E455" s="10" t="s">
-        <x:v>522</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="F455" s="10" t="s">
         <x:v>3</x:v>
@@ -18909,13 +18912,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C456" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D456" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E456" s="10" t="s">
-        <x:v>523</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="F456" s="10" t="s">
         <x:v>3</x:v>
@@ -18943,7 +18946,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="C457" s="10" t="s">
-        <x:v>513</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="D457" s="10" t="s">
         <x:v>80</x:v>
@@ -18977,13 +18980,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C458" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D458" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E458" s="10" t="s">
-        <x:v>525</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="F458" s="10" t="s">
         <x:v>3</x:v>
@@ -19011,13 +19014,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C459" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D459" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E459" s="10" t="s">
-        <x:v>526</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="F459" s="10" t="s">
         <x:v>3</x:v>
@@ -19045,13 +19048,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C460" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D460" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E460" s="10" t="s">
-        <x:v>527</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="F460" s="10" t="s">
         <x:v>3</x:v>
@@ -19079,13 +19082,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C461" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D461" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E461" s="10" t="s">
-        <x:v>528</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="F461" s="10" t="s">
         <x:v>3</x:v>
@@ -19113,13 +19116,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C462" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D462" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E462" s="10" t="s">
-        <x:v>529</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="F462" s="10" t="s">
         <x:v>3</x:v>
@@ -19147,13 +19150,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C463" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D463" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E463" s="10" t="s">
-        <x:v>530</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="F463" s="10" t="s">
         <x:v>3</x:v>
@@ -19181,13 +19184,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C464" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D464" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E464" s="10" t="s">
-        <x:v>531</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F464" s="10" t="s">
         <x:v>3</x:v>
@@ -19215,13 +19218,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C465" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D465" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E465" s="10" t="s">
-        <x:v>532</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="F465" s="10" t="s">
         <x:v>3</x:v>
@@ -19249,13 +19252,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C466" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D466" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E466" s="10" t="s">
-        <x:v>533</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="F466" s="10" t="s">
         <x:v>3</x:v>
@@ -19283,13 +19286,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C467" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D467" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E467" s="10" t="s">
-        <x:v>534</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="F467" s="10" t="s">
         <x:v>3</x:v>
@@ -19317,13 +19320,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C468" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D468" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E468" s="10" t="s">
-        <x:v>535</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="F468" s="10" t="s">
         <x:v>3</x:v>
@@ -19351,13 +19354,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C469" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D469" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E469" s="10" t="s">
-        <x:v>536</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="F469" s="10" t="s">
         <x:v>3</x:v>
@@ -19385,13 +19388,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C470" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D470" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E470" s="10" t="s">
-        <x:v>537</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="F470" s="10" t="s">
         <x:v>3</x:v>
@@ -19419,13 +19422,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C471" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D471" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E471" s="10" t="s">
-        <x:v>455</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="F471" s="10" t="s">
         <x:v>3</x:v>
@@ -19453,13 +19456,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C472" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D472" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E472" s="10" t="s">
-        <x:v>538</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="F472" s="10" t="s">
         <x:v>3</x:v>
@@ -19487,13 +19490,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C473" s="10" t="s">
-        <x:v>524</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D473" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E473" s="10" t="s">
-        <x:v>539</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="F473" s="10" t="s">
         <x:v>3</x:v>
@@ -19521,13 +19524,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C474" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D474" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E474" s="10" t="s">
-        <x:v>541</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="F474" s="10" t="s">
         <x:v>3</x:v>
@@ -19555,13 +19558,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C475" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D475" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E475" s="10" t="s">
-        <x:v>542</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="F475" s="10" t="s">
         <x:v>3</x:v>
@@ -19589,13 +19592,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C476" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D476" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E476" s="10" t="s">
-        <x:v>543</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="F476" s="10" t="s">
         <x:v>3</x:v>
@@ -19623,13 +19626,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C477" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D477" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E477" s="10" t="s">
-        <x:v>544</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="F477" s="10" t="s">
         <x:v>3</x:v>
@@ -19657,13 +19660,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C478" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D478" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E478" s="10" t="s">
-        <x:v>545</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="F478" s="10" t="s">
         <x:v>3</x:v>
@@ -19691,13 +19694,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C479" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D479" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E479" s="10" t="s">
-        <x:v>546</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="F479" s="10" t="s">
         <x:v>3</x:v>
@@ -19725,13 +19728,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C480" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D480" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E480" s="10" t="s">
-        <x:v>547</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="F480" s="10" t="s">
         <x:v>3</x:v>
@@ -19759,13 +19762,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C481" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D481" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E481" s="10" t="s">
-        <x:v>548</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="F481" s="10" t="s">
         <x:v>3</x:v>
@@ -19793,13 +19796,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C482" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D482" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E482" s="10" t="s">
-        <x:v>549</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="F482" s="10" t="s">
         <x:v>3</x:v>
@@ -19827,13 +19830,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C483" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D483" s="10" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="E483" s="10" t="s">
-        <x:v>550</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="F483" s="10" t="s">
         <x:v>3</x:v>
@@ -19861,13 +19864,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C484" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D484" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E484" s="10" t="s">
-        <x:v>551</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="F484" s="10" t="s">
         <x:v>3</x:v>
@@ -19895,13 +19898,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C485" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D485" s="10" t="s">
         <x:v>74</x:v>
       </x:c>
       <x:c r="E485" s="10" t="s">
-        <x:v>552</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="F485" s="10" t="s">
         <x:v>3</x:v>
@@ -19929,13 +19932,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C486" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D486" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E486" s="10" t="s">
-        <x:v>553</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="F486" s="10" t="s">
         <x:v>3</x:v>
@@ -19963,13 +19966,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C487" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D487" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E487" s="10" t="s">
-        <x:v>554</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="F487" s="10" t="s">
         <x:v>3</x:v>
@@ -19997,13 +20000,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C488" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D488" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E488" s="10" t="s">
-        <x:v>555</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="F488" s="10" t="s">
         <x:v>3</x:v>
@@ -20031,13 +20034,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="C489" s="10" t="s">
-        <x:v>540</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D489" s="10" t="s">
         <x:v>80</x:v>
       </x:c>
       <x:c r="E489" s="10" t="s">
-        <x:v>556</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="F489" s="10" t="s">
         <x:v>3</x:v>
@@ -20065,13 +20068,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C490" s="10" t="s">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="D490" s="10" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="E490" s="10" t="s">
         <x:v>557</x:v>
-      </x:c>
-      <x:c r="D490" s="10" t="s">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="E490" s="10" t="s">
-        <x:v>559</x:v>
       </x:c>
       <x:c r="F490" s="10" t="s">
         <x:v>3</x:v>
@@ -20099,13 +20102,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C491" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D491" s="10" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="E491" s="10" t="s">
         <x:v>558</x:v>
-      </x:c>
-      <x:c r="E491" s="10" t="s">
-        <x:v>560</x:v>
       </x:c>
       <x:c r="F491" s="10" t="s">
         <x:v>3</x:v>
@@ -20133,13 +20136,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C492" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D492" s="10" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E492" s="10" t="s">
-        <x:v>561</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="F492" s="10" t="s">
         <x:v>3</x:v>
@@ -20167,13 +20170,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C493" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D493" s="10" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E493" s="10" t="s">
-        <x:v>562</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="F493" s="10" t="s">
         <x:v>3</x:v>
@@ -20201,13 +20204,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C494" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D494" s="10" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E494" s="10" t="s">
-        <x:v>563</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="F494" s="10" t="s">
         <x:v>3</x:v>
@@ -20235,13 +20238,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C495" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D495" s="10" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E495" s="10" t="s">
-        <x:v>564</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="F495" s="10" t="s">
         <x:v>3</x:v>
@@ -20269,13 +20272,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C496" s="10" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D496" s="10" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E496" s="10" t="s">
-        <x:v>565</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="F496" s="10" t="s">
         <x:v>3</x:v>
@@ -20303,13 +20306,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C497" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D497" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E497" t="s">
-        <x:v>566</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="F497" t="s">
         <x:v>3</x:v>
@@ -20337,10 +20340,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C498" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D498" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E498" t="str">
         <x:v>Dùng đúng partition_seed=42 và membership checksum đã khóa.</x:v>
@@ -20371,10 +20374,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C499" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D499" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E499" t="str">
         <x:v>Báo cáo kết quả từng seed, mean và sample SD (ddof=1) trên 10 training_seed đã khóa.</x:v>
@@ -20405,13 +20408,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C500" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D500" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E500" t="s">
-        <x:v>567</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="F500" t="s">
         <x:v>3</x:v>
@@ -20439,13 +20442,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C501" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D501" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E501" t="s">
-        <x:v>568</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="F501" t="s">
         <x:v>3</x:v>
@@ -20473,13 +20476,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C502" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D502" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E502" t="s">
-        <x:v>569</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="F502" t="s">
         <x:v>3</x:v>
@@ -20507,13 +20510,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C503" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D503" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E503" t="s">
-        <x:v>570</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="F503" t="s">
         <x:v>3</x:v>
@@ -20541,13 +20544,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C504" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D504" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E504" t="s">
-        <x:v>571</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="F504" t="s">
         <x:v>3</x:v>
@@ -20575,13 +20578,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C505" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D505" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E505" t="s">
-        <x:v>572</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="F505" t="s">
         <x:v>3</x:v>
@@ -20609,13 +20612,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C506" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D506" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E506" t="s">
-        <x:v>573</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="F506" t="s">
         <x:v>3</x:v>
@@ -20643,10 +20646,10 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C507" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D507" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E507" t="s">
         <x:v>17</x:v>
@@ -20677,13 +20680,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C508" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D508" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E508" t="s">
-        <x:v>574</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="F508" t="s">
         <x:v>3</x:v>
@@ -20711,13 +20714,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="C509" t="s">
-        <x:v>557</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D509" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E509" t="s">
-        <x:v>575</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="F509" t="s">
         <x:v>3</x:v>
@@ -20745,13 +20748,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C510" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D510" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E510" t="s">
-        <x:v>577</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="F510" t="s">
         <x:v>3</x:v>
@@ -20779,13 +20782,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C511" t="s">
+        <x:v>574</x:v>
+      </x:c>
+      <x:c r="D511" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="E511" t="s">
         <x:v>576</x:v>
-      </x:c>
-      <x:c r="D511" t="s">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="E511" t="s">
-        <x:v>578</x:v>
       </x:c>
       <x:c r="F511" t="s">
         <x:v>3</x:v>
@@ -20813,13 +20816,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C512" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D512" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E512" t="s">
-        <x:v>579</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="F512" t="s">
         <x:v>3</x:v>
@@ -20847,13 +20850,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C513" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D513" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E513" t="s">
-        <x:v>580</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="F513" t="s">
         <x:v>3</x:v>
@@ -20881,13 +20884,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C514" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D514" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E514" t="s">
-        <x:v>581</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="F514" t="s">
         <x:v>3</x:v>
@@ -20915,13 +20918,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C515" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D515" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E515" t="s">
-        <x:v>582</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="F515" t="s">
         <x:v>3</x:v>
@@ -20949,13 +20952,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C516" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D516" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E516" t="s">
-        <x:v>583</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="F516" t="s">
         <x:v>3</x:v>
@@ -20983,13 +20986,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C517" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D517" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E517" t="s">
-        <x:v>584</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="F517" t="s">
         <x:v>3</x:v>
@@ -21017,10 +21020,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C518" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D518" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E518" t="str">
         <x:v>Không để supervised và SSL lệch partition membership, membership checksum hoặc training_seed_index.</x:v>
@@ -21051,13 +21054,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C519" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D519" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E519" t="s">
-        <x:v>585</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="F519" t="s">
         <x:v>3</x:v>
@@ -21085,10 +21088,10 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C520" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D520" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E520" t="str">
         <x:v>Không chỉ chạy một training_seed cho một experiment cell và không silently replace run lỗi bằng seed khác.</x:v>
@@ -21119,13 +21122,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C521" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D521" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E521" t="s">
-        <x:v>586</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="F521" t="s">
         <x:v>3</x:v>
@@ -21153,13 +21156,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C522" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D522" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E522" t="s">
-        <x:v>587</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="F522" t="s">
         <x:v>3</x:v>
@@ -21187,13 +21190,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C523" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D523" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E523" t="s">
-        <x:v>588</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="F523" t="s">
         <x:v>3</x:v>
@@ -21221,13 +21224,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C524" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D524" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E524" t="s">
-        <x:v>589</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="F524" t="s">
         <x:v>3</x:v>
@@ -21255,13 +21258,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C525" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D525" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E525" t="s">
-        <x:v>590</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="F525" t="s">
         <x:v>3</x:v>
@@ -21289,13 +21292,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C526" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D526" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E526" t="s">
-        <x:v>591</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="F526" t="s">
         <x:v>3</x:v>
@@ -21323,13 +21326,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C527" t="s">
-        <x:v>576</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D527" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E527" t="s">
-        <x:v>592</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="F527" t="s">
         <x:v>3</x:v>
@@ -21357,13 +21360,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C528" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D528" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E528" t="s">
-        <x:v>594</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="F528" t="s">
         <x:v>3</x:v>
@@ -21391,10 +21394,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C529" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D529" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E529" t="str">
         <x:v>So sánh supervised và SSL trên cùng partition_seed=42, cùng membership checksum và cùng training_seed_index.</x:v>
@@ -21425,10 +21428,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C530" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D530" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E530" t="str">
         <x:v>Báo cáo đủ kết quả từng seed, mean và sample SD (ddof=1) trên 10 training_seed đã khóa.</x:v>
@@ -21459,13 +21462,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C531" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="D531" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="E531" t="s">
         <x:v>593</x:v>
-      </x:c>
-      <x:c r="D531" t="s">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="E531" t="s">
-        <x:v>595</x:v>
       </x:c>
       <x:c r="F531" t="s">
         <x:v>3</x:v>
@@ -21493,13 +21496,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C532" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D532" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E532" t="s">
-        <x:v>596</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="F532" t="s">
         <x:v>3</x:v>
@@ -21527,13 +21530,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C533" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D533" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E533" t="s">
-        <x:v>597</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="F533" t="s">
         <x:v>3</x:v>
@@ -21561,13 +21564,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="C534" t="s">
-        <x:v>593</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="D534" t="s">
-        <x:v>558</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E534" t="s">
-        <x:v>598</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="F534" t="s">
         <x:v>3</x:v>
@@ -26906,7 +26909,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b5fe4a224d54516"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2192d610e7c6426b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27379,7 +27382,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b10ca77510e41ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2273c62c6da4acd"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>